<commit_message>
docs(qa): record substack chat handoff pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Ree3148a5fd9e4321"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R95e3f7b0aaf54c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R2028ffdb3ee548af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R84600a3de069482b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rb7e0eb095b794ba1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rb03963a071854132"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R63637a88dd99415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rd1b2ae36500e46e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1917,31 +1917,77 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
-      <x:c r="A20" s="14"/>
-      <x:c r="B20" s="14"/>
-      <x:c r="C20" s="14"/>
-      <x:c r="D20" s="14"/>
-      <x:c r="E20" s="14"/>
-      <x:c r="F20" s="14"/>
-      <x:c r="G20" s="14"/>
-      <x:c r="H20" s="14"/>
-      <x:c r="I20" s="14"/>
-      <x:c r="J20" s="14"/>
-      <x:c r="K20" s="14"/>
-      <x:c r="L20" s="14"/>
-      <x:c r="M20" s="14"/>
-      <x:c r="N20" s="14"/>
-      <x:c r="O20" s="14"/>
-      <x:c r="P20" s="14"/>
-      <x:c r="Q20" s="14"/>
-      <x:c r="R20" s="14"/>
-      <x:c r="S20" s="14"/>
-      <x:c r="T20" s="14"/>
-      <x:c r="U20" s="14"/>
-      <x:c r="V20" s="14"/>
-      <x:c r="W20" s="14"/>
-      <x:c r="X20" s="14"/>
-      <x:c r="Y20" s="14"/>
+      <x:c r="A20" s="14" t="str">
+        <x:v>F-019</x:v>
+      </x:c>
+      <x:c r="B20" s="14" t="str">
+        <x:v>Substack Chat Reply Destination</x:v>
+      </x:c>
+      <x:c r="C20" s="14" t="str">
+        <x:v>Membership / Access Copy</x:v>
+      </x:c>
+      <x:c r="D20" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E20" s="14" t="str">
+        <x:v>Join handoff copy across site and README</x:v>
+      </x:c>
+      <x:c r="F20" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G20" s="14" t="str">
+        <x:v>As a prospective member, I want one concrete place to send my GitHub details so that I do not have to guess where to reply after joining.</x:v>
+      </x:c>
+      <x:c r="H20" s="14" t="str">
+        <x:v>The public repo should explicitly say to send the GitHub username or account email through Substack Chat after joining.</x:v>
+      </x:c>
+      <x:c r="I20" s="14" t="str">
+        <x:v>Code inspection confirms the join strip, access steps, member note, join-links panel, and README now point members to Substack Chat as the handoff destination for GitHub details.</x:v>
+      </x:c>
+      <x:c r="J20" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K20" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L20" s="14" t="str">
+        <x:v>Inspect src/app.js and README.md for the join handoff copy and confirm Substack Chat is named as the concrete reply destination.</x:v>
+      </x:c>
+      <x:c r="M20" s="14" t="str">
+        <x:v>Pass - the reply destination is now explicit and consistent across the public site and README.</x:v>
+      </x:c>
+      <x:c r="N20" s="14" t="str"/>
+      <x:c r="O20" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P20" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q20" s="14" t="str"/>
+      <x:c r="R20" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S20" s="14" t="str">
+        <x:v>df25d10</x:v>
+      </x:c>
+      <x:c r="T20" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new Substack Chat row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U20" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after setting Substack Chat as the join handoff destination.</x:v>
+      </x:c>
+      <x:c r="V20" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W20" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X20" s="14" t="str">
+        <x:v>This row captures the move from ambiguous reply wording to one concrete Substack Chat destination.</x:v>
+      </x:c>
+      <x:c r="Y20" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="14"/>
@@ -12265,7 +12311,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12281,7 +12327,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12345,14 +12391,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record x contact path pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rb7e0eb095b794ba1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rb03963a071854132"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R63637a88dd99415d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rd1b2ae36500e46e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R56e83c32525d4fe6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rb32be5526ed94f00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R8965438b62744d8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R3d6d8cfeaf1346d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1990,31 +1990,77 @@
       </x:c>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="14"/>
-      <x:c r="B21" s="14"/>
-      <x:c r="C21" s="14"/>
-      <x:c r="D21" s="14"/>
-      <x:c r="E21" s="14"/>
-      <x:c r="F21" s="14"/>
-      <x:c r="G21" s="14"/>
-      <x:c r="H21" s="14"/>
-      <x:c r="I21" s="14"/>
-      <x:c r="J21" s="14"/>
-      <x:c r="K21" s="14"/>
-      <x:c r="L21" s="14"/>
-      <x:c r="M21" s="14"/>
-      <x:c r="N21" s="14"/>
-      <x:c r="O21" s="14"/>
-      <x:c r="P21" s="14"/>
-      <x:c r="Q21" s="14"/>
-      <x:c r="R21" s="14"/>
-      <x:c r="S21" s="14"/>
-      <x:c r="T21" s="14"/>
-      <x:c r="U21" s="14"/>
-      <x:c r="V21" s="14"/>
-      <x:c r="W21" s="14"/>
-      <x:c r="X21" s="14"/>
-      <x:c r="Y21" s="14"/>
+      <x:c r="A21" s="14" t="str">
+        <x:v>F-020</x:v>
+      </x:c>
+      <x:c r="B21" s="14" t="str">
+        <x:v>Alternate X Contact Path</x:v>
+      </x:c>
+      <x:c r="C21" s="14" t="str">
+        <x:v>Membership / Access Copy</x:v>
+      </x:c>
+      <x:c r="D21" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E21" s="14" t="str">
+        <x:v>Join strip, join steps, join links panel, access-flow panel, README access section</x:v>
+      </x:c>
+      <x:c r="F21" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G21" s="14" t="str">
+        <x:v>As a prospective member, I want an alternate direct-message path so that I can still send my GitHub details even if I prefer X over Substack Chat.</x:v>
+      </x:c>
+      <x:c r="H21" s="14" t="str">
+        <x:v>The public repo should include X @AITrailblazerQ as an additional DM route for sending GitHub details, while preserving the existing Substack Chat path and invite flow.</x:v>
+      </x:c>
+      <x:c r="I21" s="14" t="str">
+        <x:v>Code inspection confirms the join strip, join steps, member note, join links panel, access-flow panel, and README now include X @AITrailblazerQ as an additional contact path for private access handoff.</x:v>
+      </x:c>
+      <x:c r="J21" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K21" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L21" s="14" t="str">
+        <x:v>Inspect src/app.js and README.md for the join handoff copy and confirm X @AITrailblazerQ is included as an additional DM path alongside Substack Chat.</x:v>
+      </x:c>
+      <x:c r="M21" s="14" t="str">
+        <x:v>Pass - the public site and README now present X as an alternate contact route without changing the rest of the private-repo access flow.</x:v>
+      </x:c>
+      <x:c r="N21" s="14" t="str"/>
+      <x:c r="O21" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P21" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q21" s="14" t="str"/>
+      <x:c r="R21" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S21" s="14" t="str">
+        <x:v>8c98d9e</x:v>
+      </x:c>
+      <x:c r="T21" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new X contact row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U21" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after adding the X contact path for private-access handoff.</x:v>
+      </x:c>
+      <x:c r="V21" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W21" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X21" s="14" t="str">
+        <x:v>This row captures the addition of the AITrailblazerQ X account as an alternate private-access contact path.</x:v>
+      </x:c>
+      <x:c r="Y21" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="14"/>
@@ -12311,7 +12357,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12327,7 +12373,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12391,14 +12437,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record subscribe path pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rb8d8a4a48f2e4e82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R5844e1a13cc44ae1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rb9a8e0d939904b11"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R9094e3314b904895"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R7b20f3316d834545"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rf9185639ef454010"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Raad2983096684c34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rf2774d4d75e24ca5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2136,31 +2136,77 @@
       </x:c>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="14"/>
-      <x:c r="B23" s="14"/>
-      <x:c r="C23" s="14"/>
-      <x:c r="D23" s="14"/>
-      <x:c r="E23" s="14"/>
-      <x:c r="F23" s="14"/>
-      <x:c r="G23" s="14"/>
-      <x:c r="H23" s="14"/>
-      <x:c r="I23" s="14"/>
-      <x:c r="J23" s="14"/>
-      <x:c r="K23" s="14"/>
-      <x:c r="L23" s="14"/>
-      <x:c r="M23" s="14"/>
-      <x:c r="N23" s="14"/>
-      <x:c r="O23" s="14"/>
-      <x:c r="P23" s="14"/>
-      <x:c r="Q23" s="14"/>
-      <x:c r="R23" s="14"/>
-      <x:c r="S23" s="14"/>
-      <x:c r="T23" s="14"/>
-      <x:c r="U23" s="14"/>
-      <x:c r="V23" s="14"/>
-      <x:c r="W23" s="14"/>
-      <x:c r="X23" s="14"/>
-      <x:c r="Y23" s="14"/>
+      <x:c r="A23" s="14" t="str">
+        <x:v>F-022</x:v>
+      </x:c>
+      <x:c r="B23" s="14" t="str">
+        <x:v>Subscribe Page As Primary Join Path</x:v>
+      </x:c>
+      <x:c r="C23" s="14" t="str">
+        <x:v>Membership / Conversion</x:v>
+      </x:c>
+      <x:c r="D23" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E23" s="14" t="str">
+        <x:v>Hero primary CTA, join strip, join links panel, access-flow panel, README access section</x:v>
+      </x:c>
+      <x:c r="F23" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G23" s="14" t="str">
+        <x:v>As a prospective member, I want the main Alpha link to take me to the actual subscription page so that I can subscribe immediately instead of landing on an explainer first.</x:v>
+      </x:c>
+      <x:c r="H23" s="14" t="str">
+        <x:v>The public repo should use DeltaSignal's `/subscribe` page as the main join destination, while keeping the Alpha Circle note as an explainer link for visitors who want context first.</x:v>
+      </x:c>
+      <x:c r="I23" s="14" t="str">
+        <x:v>Code inspection confirms the hero CTA, join strip, join links panel, access-flow panel, and README now use the DeltaSignal subscribe page as the primary join destination and keep the Alpha Circle note as a secondary explainer link.</x:v>
+      </x:c>
+      <x:c r="J23" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K23" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L23" s="14" t="str">
+        <x:v>Inspect src/app.js and README.md for the primary Alpha-link targets and confirm the subscribe-page URL is now the main membership destination.</x:v>
+      </x:c>
+      <x:c r="M23" s="14" t="str">
+        <x:v>Pass - the public repo now points its main conversion path to the actual DeltaSignal subscribe page instead of the explainer note.</x:v>
+      </x:c>
+      <x:c r="N23" s="14" t="str"/>
+      <x:c r="O23" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P23" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q23" s="14" t="str"/>
+      <x:c r="R23" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S23" s="14" t="str">
+        <x:v>0fa1929</x:v>
+      </x:c>
+      <x:c r="T23" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new subscribe-path row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U23" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after restoring the subscribe page as the main Alpha join path.</x:v>
+      </x:c>
+      <x:c r="V23" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W23" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X23" s="14" t="str">
+        <x:v>This row captures the restoration of the public repo's main Alpha join path to the actual DeltaSignal subscribe page.</x:v>
+      </x:c>
+      <x:c r="Y23" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="14"/>
@@ -12403,7 +12449,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12419,7 +12465,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12483,14 +12529,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record operator alpha link pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R7b20f3316d834545"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rf9185639ef454010"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Raad2983096684c34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rf2774d4d75e24ca5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rbaabe2c39fef4156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R5cb1daefd2514cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R679bff087afc49ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rc560b54914f04c0a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2209,31 +2209,77 @@
       </x:c>
     </x:row>
     <x:row r="24">
-      <x:c r="A24" s="14"/>
-      <x:c r="B24" s="14"/>
-      <x:c r="C24" s="14"/>
-      <x:c r="D24" s="14"/>
-      <x:c r="E24" s="14"/>
-      <x:c r="F24" s="14"/>
-      <x:c r="G24" s="14"/>
-      <x:c r="H24" s="14"/>
-      <x:c r="I24" s="14"/>
-      <x:c r="J24" s="14"/>
-      <x:c r="K24" s="14"/>
-      <x:c r="L24" s="14"/>
-      <x:c r="M24" s="14"/>
-      <x:c r="N24" s="14"/>
-      <x:c r="O24" s="14"/>
-      <x:c r="P24" s="14"/>
-      <x:c r="Q24" s="14"/>
-      <x:c r="R24" s="14"/>
-      <x:c r="S24" s="14"/>
-      <x:c r="T24" s="14"/>
-      <x:c r="U24" s="14"/>
-      <x:c r="V24" s="14"/>
-      <x:c r="W24" s="14"/>
-      <x:c r="X24" s="14"/>
-      <x:c r="Y24" s="14"/>
+      <x:c r="A24" s="14" t="str">
+        <x:v>F-023</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>Operator-Specified Alpha Link</x:v>
+      </x:c>
+      <x:c r="C24" s="14" t="str">
+        <x:v>Membership / Conversion</x:v>
+      </x:c>
+      <x:c r="D24" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E24" s="14" t="str">
+        <x:v>Hero primary CTA, join strip, join links panel, access-flow panel, README access section</x:v>
+      </x:c>
+      <x:c r="F24" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G24" s="14" t="str">
+        <x:v>As a prospective member, I want the public repo to use the exact Alpha link chosen by the operator so that the join path matches the intended campaign destination.</x:v>
+      </x:c>
+      <x:c r="H24" s="14" t="str">
+        <x:v>The public repo should use `https://substack.com/@deltasignalai/p-179433731` as the primary Alpha path in the main CTA and access instructions, while leaving the GitHub-detail handoff flow unchanged.</x:v>
+      </x:c>
+      <x:c r="I24" s="14" t="str">
+        <x:v>Code inspection confirms the hero CTA, join strip, join links panel, access-flow panel, and README now use the operator-specified Alpha Circle note as the primary join destination.</x:v>
+      </x:c>
+      <x:c r="J24" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K24" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L24" s="14" t="str">
+        <x:v>Inspect src/app.js and README.md for the primary Alpha-link targets and confirm the operator-specified note URL is now the main membership destination.</x:v>
+      </x:c>
+      <x:c r="M24" s="14" t="str">
+        <x:v>Pass - the public repo now uses the exact Alpha URL specified by the operator as its main join path.</x:v>
+      </x:c>
+      <x:c r="N24" s="14" t="str"/>
+      <x:c r="O24" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P24" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q24" s="14" t="str"/>
+      <x:c r="R24" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S24" s="14" t="str">
+        <x:v>97481f3</x:v>
+      </x:c>
+      <x:c r="T24" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new operator-link row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U24" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after switching the main Alpha path back to the operator-specified URL.</x:v>
+      </x:c>
+      <x:c r="V24" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W24" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X24" s="14" t="str">
+        <x:v>This row captures the switch back to the operator-specified Alpha Circle link.</x:v>
+      </x:c>
+      <x:c r="Y24" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="14"/>
@@ -12449,7 +12495,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12465,7 +12511,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12529,14 +12575,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record substack-only handoff pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rbaabe2c39fef4156"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R5cb1daefd2514cfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R679bff087afc49ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rc560b54914f04c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Ra6e78d0b26e640f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R9fd53acceeb8433c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R7d0f1e5478f74e7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R5961d0e369e34f08"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2282,31 +2282,77 @@
       </x:c>
     </x:row>
     <x:row r="25">
-      <x:c r="A25" s="14"/>
-      <x:c r="B25" s="14"/>
-      <x:c r="C25" s="14"/>
-      <x:c r="D25" s="14"/>
-      <x:c r="E25" s="14"/>
-      <x:c r="F25" s="14"/>
-      <x:c r="G25" s="14"/>
-      <x:c r="H25" s="14"/>
-      <x:c r="I25" s="14"/>
-      <x:c r="J25" s="14"/>
-      <x:c r="K25" s="14"/>
-      <x:c r="L25" s="14"/>
-      <x:c r="M25" s="14"/>
-      <x:c r="N25" s="14"/>
-      <x:c r="O25" s="14"/>
-      <x:c r="P25" s="14"/>
-      <x:c r="Q25" s="14"/>
-      <x:c r="R25" s="14"/>
-      <x:c r="S25" s="14"/>
-      <x:c r="T25" s="14"/>
-      <x:c r="U25" s="14"/>
-      <x:c r="V25" s="14"/>
-      <x:c r="W25" s="14"/>
-      <x:c r="X25" s="14"/>
-      <x:c r="Y25" s="14"/>
+      <x:c r="A25" s="14" t="str">
+        <x:v>F-024</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>Substack-Only Access Handoff</x:v>
+      </x:c>
+      <x:c r="C25" s="14" t="str">
+        <x:v>Membership / Access Copy</x:v>
+      </x:c>
+      <x:c r="D25" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E25" s="14" t="str">
+        <x:v>Join strip, join steps, join links panel, access-flow panel, README access section</x:v>
+      </x:c>
+      <x:c r="F25" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G25" s="14" t="str">
+        <x:v>As a prospective member, I want one single DM handoff path so that I know exactly where to send my GitHub details after joining.</x:v>
+      </x:c>
+      <x:c r="H25" s="14" t="str">
+        <x:v>The public repo should use Substack Chat as the only GitHub-details handoff path and remove the X DM option from the access copy.</x:v>
+      </x:c>
+      <x:c r="I25" s="14" t="str">
+        <x:v>Code inspection confirms the join strip, join steps, member note, access-flow panel, and README now point only to Substack Chat for the GitHub-details handoff.</x:v>
+      </x:c>
+      <x:c r="J25" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K25" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L25" s="14" t="str">
+        <x:v>Inspect src/app.js and README.md for the access handoff copy and confirm X DM references are removed while Substack Chat remains.</x:v>
+      </x:c>
+      <x:c r="M25" s="14" t="str">
+        <x:v>Pass - the public site and README now use Substack Chat as the only DM path for GitHub-access handoff.</x:v>
+      </x:c>
+      <x:c r="N25" s="14" t="str"/>
+      <x:c r="O25" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P25" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q25" s="14" t="str"/>
+      <x:c r="R25" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S25" s="14" t="str">
+        <x:v>1a43b6e</x:v>
+      </x:c>
+      <x:c r="T25" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new Substack-only row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U25" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after simplifying the GitHub-access handoff to Substack Chat only.</x:v>
+      </x:c>
+      <x:c r="V25" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W25" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X25" s="14" t="str">
+        <x:v>This row captures the simplification of the public access handoff to Substack Chat only.</x:v>
+      </x:c>
+      <x:c r="Y25" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="14"/>
@@ -12495,7 +12541,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12511,7 +12557,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12575,14 +12621,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record hero access wording pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Ra6e78d0b26e640f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R9fd53acceeb8433c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R7d0f1e5478f74e7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R5961d0e369e34f08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R71f743c708424a6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R9fd296f6f2f84d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R12ad10fc83184776"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rf3d9ce375fc140ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2355,31 +2355,77 @@
       </x:c>
     </x:row>
     <x:row r="26">
-      <x:c r="A26" s="14"/>
-      <x:c r="B26" s="14"/>
-      <x:c r="C26" s="14"/>
-      <x:c r="D26" s="14"/>
-      <x:c r="E26" s="14"/>
-      <x:c r="F26" s="14"/>
-      <x:c r="G26" s="14"/>
-      <x:c r="H26" s="14"/>
-      <x:c r="I26" s="14"/>
-      <x:c r="J26" s="14"/>
-      <x:c r="K26" s="14"/>
-      <x:c r="L26" s="14"/>
-      <x:c r="M26" s="14"/>
-      <x:c r="N26" s="14"/>
-      <x:c r="O26" s="14"/>
-      <x:c r="P26" s="14"/>
-      <x:c r="Q26" s="14"/>
-      <x:c r="R26" s="14"/>
-      <x:c r="S26" s="14"/>
-      <x:c r="T26" s="14"/>
-      <x:c r="U26" s="14"/>
-      <x:c r="V26" s="14"/>
-      <x:c r="W26" s="14"/>
-      <x:c r="X26" s="14"/>
-      <x:c r="Y26" s="14"/>
+      <x:c r="A26" s="14" t="str">
+        <x:v>F-025</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>Hero Access Step Clarity</x:v>
+      </x:c>
+      <x:c r="C26" s="14" t="str">
+        <x:v>Membership / Access Copy</x:v>
+      </x:c>
+      <x:c r="D26" s="14" t="str">
+        <x:v>src/app.js</x:v>
+      </x:c>
+      <x:c r="E26" s="14" t="str">
+        <x:v>Hero access panel step 1</x:v>
+      </x:c>
+      <x:c r="F26" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G26" s="14" t="str">
+        <x:v>As a prospective member, I want the first access step described accurately so that I understand the Alpha note is the guide and the GitHub handoff still happens separately.</x:v>
+      </x:c>
+      <x:c r="H26" s="14" t="str">
+        <x:v>The hero access panel should describe the Alpha Circle note as the join guide and explain that the Substack Chat handoff is the next step for GitHub access.</x:v>
+      </x:c>
+      <x:c r="I26" s="14" t="str">
+        <x:v>Code inspection confirms the first hero access step now describes the Alpha note as the join guide and explicitly points readers to the Substack Chat handoff for GitHub invite details.</x:v>
+      </x:c>
+      <x:c r="J26" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K26" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L26" s="14" t="str">
+        <x:v>Inspect the hero access panel step 1 in src/app.js and confirm the wording no longer claims the note itself is the membership gateway.</x:v>
+      </x:c>
+      <x:c r="M26" s="14" t="str">
+        <x:v>Pass - the hero access step now describes the Alpha note as guidance rather than the gateway itself.</x:v>
+      </x:c>
+      <x:c r="N26" s="14" t="str"/>
+      <x:c r="O26" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P26" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q26" s="14" t="str"/>
+      <x:c r="R26" s="14" t="str">
+        <x:v>src/app.js, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S26" s="14" t="str">
+        <x:v>7e3190e</x:v>
+      </x:c>
+      <x:c r="T26" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new hero-copy row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U26" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after correcting the first hero access step wording.</x:v>
+      </x:c>
+      <x:c r="V26" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W26" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X26" s="14" t="str">
+        <x:v>This row captures the wording correction for the first hero access step.</x:v>
+      </x:c>
+      <x:c r="Y26" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="14"/>
@@ -12541,7 +12587,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12557,7 +12603,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12621,14 +12667,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record positioning refresh pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rf8f12ba5d0284430"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rcb8c2c91876f4b57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rf873444b96e544d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R421ea8b4f1174600"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R4d3de0ff9ed4441d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R17c83812e3684e5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Re0388b8b2d594e2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Ra61978f1955f4ef2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2501,31 +2501,77 @@
       </x:c>
     </x:row>
     <x:row r="28">
-      <x:c r="A28" s="14"/>
-      <x:c r="B28" s="14"/>
-      <x:c r="C28" s="14"/>
-      <x:c r="D28" s="14"/>
-      <x:c r="E28" s="14"/>
-      <x:c r="F28" s="14"/>
-      <x:c r="G28" s="14"/>
-      <x:c r="H28" s="14"/>
-      <x:c r="I28" s="14"/>
-      <x:c r="J28" s="14"/>
-      <x:c r="K28" s="14"/>
-      <x:c r="L28" s="14"/>
-      <x:c r="M28" s="14"/>
-      <x:c r="N28" s="14"/>
-      <x:c r="O28" s="14"/>
-      <x:c r="P28" s="14"/>
-      <x:c r="Q28" s="14"/>
-      <x:c r="R28" s="14"/>
-      <x:c r="S28" s="14"/>
-      <x:c r="T28" s="14"/>
-      <x:c r="U28" s="14"/>
-      <x:c r="V28" s="14"/>
-      <x:c r="W28" s="14"/>
-      <x:c r="X28" s="14"/>
-      <x:c r="Y28" s="14"/>
+      <x:c r="A28" s="14" t="str">
+        <x:v>F-027</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>Landing Page Positioning Refresh</x:v>
+      </x:c>
+      <x:c r="C28" s="14" t="str">
+        <x:v>Marketing / Positioning Copy</x:v>
+      </x:c>
+      <x:c r="D28" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E28" s="14" t="str">
+        <x:v>Hero copy, who-it's-for framing, value proposition cards, Alpha member benefits, README intro</x:v>
+      </x:c>
+      <x:c r="F28" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G28" s="14" t="str">
+        <x:v>As a prospective member, I want the public page to explain ATLAS-7 clearly and specifically so that I understand what it is, who it is for, and what Alpha membership unlocks.</x:v>
+      </x:c>
+      <x:c r="H28" s="14" t="str">
+        <x:v>The public landing page should present a stronger headline, a clearer value proposition, a more specific who-it's-for section, and a more concrete member-benefit summary without relying on unsupported promises.</x:v>
+      </x:c>
+      <x:c r="I28" s="14" t="str">
+        <x:v>Code inspection confirms the hero, benefit cards, Alpha section, MCP framing, and README now present a stronger positioning narrative with more specific audience and benefit language.</x:v>
+      </x:c>
+      <x:c r="J28" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K28" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L28" s="14" t="str">
+        <x:v>Inspect src/app.js and README.md for the updated headline, value proposition, audience framing, and Alpha-member benefit copy.</x:v>
+      </x:c>
+      <x:c r="M28" s="14" t="str">
+        <x:v>Pass - the public page now communicates the ATLAS-7 offer more clearly and more directly.</x:v>
+      </x:c>
+      <x:c r="N28" s="14" t="str"/>
+      <x:c r="O28" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P28" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q28" s="14" t="str"/>
+      <x:c r="R28" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S28" s="14" t="str">
+        <x:v>d6e0d6f</x:v>
+      </x:c>
+      <x:c r="T28" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new positioning row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U28" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after strengthening the public landing page positioning.</x:v>
+      </x:c>
+      <x:c r="V28" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W28" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X28" s="14" t="str">
+        <x:v>This row captures the stronger public positioning refresh for the ATLAS-7 landing page.</x:v>
+      </x:c>
+      <x:c r="Y28" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="14"/>
@@ -12633,7 +12679,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12649,7 +12695,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12713,14 +12759,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
docs(qa): record playbook 001 flagship pass
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rea3d7a1542314d78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R3067fd68c8ac42f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R991255192d73451d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R795cda8671e44288"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R79fcc4061d354b4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R11280bf8c5824c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rbb92a48f44624d30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rf64e87ae3293400e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2647,31 +2647,77 @@
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="14"/>
-      <x:c r="B30" s="14"/>
-      <x:c r="C30" s="14"/>
-      <x:c r="D30" s="14"/>
-      <x:c r="E30" s="14"/>
-      <x:c r="F30" s="14"/>
-      <x:c r="G30" s="14"/>
-      <x:c r="H30" s="14"/>
-      <x:c r="I30" s="14"/>
-      <x:c r="J30" s="14"/>
-      <x:c r="K30" s="14"/>
-      <x:c r="L30" s="14"/>
-      <x:c r="M30" s="14"/>
-      <x:c r="N30" s="14"/>
-      <x:c r="O30" s="14"/>
-      <x:c r="P30" s="14"/>
-      <x:c r="Q30" s="14"/>
-      <x:c r="R30" s="14"/>
-      <x:c r="S30" s="14"/>
-      <x:c r="T30" s="14"/>
-      <x:c r="U30" s="14"/>
-      <x:c r="V30" s="14"/>
-      <x:c r="W30" s="14"/>
-      <x:c r="X30" s="14"/>
-      <x:c r="Y30" s="14"/>
+      <x:c r="A30" s="14" t="str">
+        <x:v>F-029</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>Playbook 001 Flagship Framing</x:v>
+      </x:c>
+      <x:c r="C30" s="14" t="str">
+        <x:v>Marketing / Flagship Positioning</x:v>
+      </x:c>
+      <x:c r="D30" s="14" t="str">
+        <x:v>src/app.js, README.md</x:v>
+      </x:c>
+      <x:c r="E30" s="14" t="str">
+        <x:v>Hero message, Playbook 001 section, README intro</x:v>
+      </x:c>
+      <x:c r="F30" s="14" t="str">
+        <x:v>Visitor</x:v>
+      </x:c>
+      <x:c r="G30" s="14" t="str">
+        <x:v>As a visitor, I want the public site to make Playbook 001, the spreadsheet-first tracker, and the QA loop feel central so that I immediately understand what the repo's most important recent operating inventions are and why they matter.</x:v>
+      </x:c>
+      <x:c r="H30" s="14" t="str">
+        <x:v>The public page should prominently explain that Playbook 001 packages the spreadsheet-first tracker and Feature QA Loop, show why that method matters for trustworthy agent work, and align the README with the same thesis.</x:v>
+      </x:c>
+      <x:c r="I30" s="14" t="str">
+        <x:v>Code inspection confirms the hero now leads with the spreadsheet-first tracker and QA loop, the page includes a dedicated Playbook 001 section explaining the method and its importance, and the README mirrors that framing.</x:v>
+      </x:c>
+      <x:c r="J30" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K30" s="14" t="str">
+        <x:v>Code inspection</x:v>
+      </x:c>
+      <x:c r="L30" s="14" t="str">
+        <x:v>Inspect src/app.js for the rewritten hero, the new Playbook 001 section, and the updated contents links; inspect README.md for the matching Playbook 001 framing.</x:v>
+      </x:c>
+      <x:c r="M30" s="14" t="str">
+        <x:v>Pass - the public repo now treats Playbook 001 and its spreadsheet-plus-loop method as the flagship operating thesis instead of a background detail.</x:v>
+      </x:c>
+      <x:c r="N30" s="14" t="str"/>
+      <x:c r="O30" s="14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="P30" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q30" s="14" t="str"/>
+      <x:c r="R30" s="14" t="str">
+        <x:v>src/app.js, README.md, CHANGELOG.md, feature_status_tracker.csv</x:v>
+      </x:c>
+      <x:c r="S30" s="14" t="str">
+        <x:v>c6b17ad</x:v>
+      </x:c>
+      <x:c r="T30" s="14" t="str">
+        <x:v>Rebuild the Lit bundle, regenerate workbook and report, and confirm the new flagship-framing row is reflected in the repo QA outputs.</x:v>
+      </x:c>
+      <x:c r="U30" s="14" t="str">
+        <x:v>Pass - Lit bundle, workbook, and report regenerated successfully after promoting Playbook 001 and its spreadsheet-plus-loop method on the public landing page.</x:v>
+      </x:c>
+      <x:c r="V30" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W30" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X30" s="14" t="str">
+        <x:v>This row captures the pass that promotes Playbook 001 and explains why the spreadsheet-first tracker and the QA loop matter.</x:v>
+      </x:c>
+      <x:c r="Y30" s="14" t="str">
+        <x:v>use /goal go over every single feature and create a user story with expected behaviour based on the code keep a single canonical spreadsheet tracking the features status when done switch loop to testing every user story and documenting all errors when done fix every logistical error or ux error test every user behaviour again post fix</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="14"/>
@@ -12725,7 +12771,7 @@
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f>COUNTA('Tracker'!$A$2:$A$400)</x:f>
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
@@ -12741,7 +12787,7 @@
       </x:c>
       <x:c r="B5" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$J$2:$J$400,"Verified")</x:f>
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
@@ -12805,14 +12851,14 @@
       </x:c>
       <x:c r="B9" s="21" t="n">
         <x:f>COUNTIF('Tracker'!$V$2:$V$400,"Verified")</x:f>
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
         <x:f>COUNTA('Tracker'!$S$2:$S$400)</x:f>
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>